<commit_message>
Updated data provider files
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\IdeaProjects\APIRestAssuredProjectDemo\TestData\"/>
     </mc:Choice>
@@ -16,7 +16,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>name</t>
   </si>
@@ -53,38 +53,28 @@
     <t>id</t>
   </si>
   <si>
-    <t>Lion king Jungle</t>
-  </si>
-  <si>
-    <t>Elizabeth Queen</t>
-  </si>
-  <si>
-    <t>John Cena</t>
-  </si>
-  <si>
-    <t>axzbcd123vbg@gmail.com</t>
-  </si>
-  <si>
-    <t>234fgh123mnb@gmail.com</t>
-  </si>
-  <si>
-    <t>lmn3vcxvb@gmail.com</t>
-  </si>
-  <si>
-    <t>1021</t>
-  </si>
-  <si>
-    <t>1022</t>
-  </si>
-  <si>
-    <t>1023</t>
+    <t>J John Cena</t>
+  </si>
+  <si>
+    <t>AElizabeth Queen</t>
+  </si>
+  <si>
+    <t>ELion king Jungle</t>
+  </si>
+  <si>
+    <t>234123john@gmail.com</t>
+  </si>
+  <si>
+    <t>2345queen@gmail.com</t>
+  </si>
+  <si>
+    <t>54678king@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -438,8 +428,8 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="15.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -461,7 +451,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>
@@ -471,9 +461,6 @@
       </c>
       <c r="D2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -489,13 +476,10 @@
       <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" t="s" s="0">
-        <v>16</v>
-      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>14</v>
@@ -505,9 +489,6 @@
       </c>
       <c r="D4" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Error scenario testcases
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\IdeaProjects\APIRestAssuredProjectDemo\TestData\"/>
     </mc:Choice>
@@ -16,7 +16,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>name</t>
   </si>
@@ -69,12 +69,22 @@
   </si>
   <si>
     <t>54678king@gmail.com</t>
+  </si>
+  <si>
+    <t>1022</t>
+  </si>
+  <si>
+    <t>1023</t>
+  </si>
+  <si>
+    <t>1024</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -428,8 +438,8 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="15.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="19.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -462,6 +472,9 @@
       <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="E2" t="s" s="0">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -476,6 +489,9 @@
       <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="E3" t="s" s="0">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -489,6 +505,9 @@
       </c>
       <c r="D4" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>